<commit_message>
CLEAN UP POLLOCK SCRIPTS
</commit_message>
<xml_diff>
--- a/GOA pollock/Data/GOA_25_pollock_single_species_1970-2024.xlsx
+++ b/GOA pollock/Data/GOA_25_pollock_single_species_1970-2024.xlsx
@@ -1189,8 +1189,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Composition weights for composition likelihood. _x000D_
-After running model, these will update to McAllister &amp; Ianelli 1997 weights using the harmonic mean.</t>
+          <t>Composition weight, on a scale set by 'Comp_distribution'. _x000D_
+Under a multinomial it is the natural-scale multiplier on the input sample size. _x000D_
+Under a Dirichlet-multinomial the model uses exp(Comp_weights), so the column is the LOG of the starting weight -- the usual template value of 1 is a starting weight of e, not 1; use 0 for a weight of 1. _x000D_
+Read when a model is built from scratch -- a refit keeps the weight it is given. _x000D_
+See 'Comp_weights_mcallister' for the weight a fit implies, and reweight_comps() to tune towards it.</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1229,10 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Composition weights for CAAL  likelihood.</t>
+          <t>Conditional age-at-length composition weight, on a scale set by 'CAAL_distribution' (as for 'Comp_weights'). _x000D_
+Under a multinomial it is the natural-scale multiplier on the input sample size. _x000D_
+Under a Dirichlet-multinomial the model uses exp(CAAL_weights), so the column is the LOG of the starting weight -- the default of 1 is a starting weight of e, not 1. _x000D_
+Read when a model is built from scratch -- a refit keeps the weight it is given.</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1934,10 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Diet composition weight (multinomial multiplier) per predator species.</t>
+          <t>Diet composition weight per predator species, on a scale set by 'Diet_distribution' (as for 'Comp_weights'). _x000D_
+Under a multinomial it is the natural-scale multiplier on the input sample size. _x000D_
+Under a Dirichlet-multinomial the model uses exp(Diet_comp_weights), so the column is the LOG of the starting weight. _x000D_
+Read when a model is built from scratch -- a refit keeps the weight it is given.</t>
         </is>
       </c>
     </row>
@@ -32417,7 +32426,7 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>0.06173061730617306</v>
+        <v>0.06173061730617307</v>
       </c>
       <c r="L3">
         <v>0.1206112061120611</v>
@@ -32432,7 +32441,7 @@
         <v>0.04460044600446005</v>
       </c>
       <c r="P3">
-        <v>0.05936059360593606</v>
+        <v>0.05936059360593607</v>
       </c>
       <c r="Q3">
         <v>0.06451064510645106</v>
@@ -32475,7 +32484,7 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>0.0971009710097101</v>
+        <v>0.09710097100971012</v>
       </c>
       <c r="L4">
         <v>0.06252062520625207</v>
@@ -32487,13 +32496,13 @@
         <v>0.1646116461164612</v>
       </c>
       <c r="O4">
-        <v>0.08367083670836707</v>
+        <v>0.08367083670836709</v>
       </c>
       <c r="P4">
-        <v>0.05362053620536205</v>
+        <v>0.05362053620536206</v>
       </c>
       <c r="Q4">
-        <v>0.08754087540875409</v>
+        <v>0.0875408754087541</v>
       </c>
       <c r="R4">
         <v>0.1456014560145601</v>
@@ -32649,10 +32658,10 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>0.7731845363092739</v>
+        <v>0.7731845363092738</v>
       </c>
       <c r="L7">
-        <v>0.04965900681986361</v>
+        <v>0.0496590068198636</v>
       </c>
       <c r="M7">
         <v>0.01142977140457191</v>
@@ -32661,16 +32670,16 @@
         <v>0.02731945361092778</v>
       </c>
       <c r="O7">
-        <v>0.03208935821283575</v>
+        <v>0.03208935821283574</v>
       </c>
       <c r="P7">
-        <v>0.06050878982420353</v>
+        <v>0.06050878982420351</v>
       </c>
       <c r="Q7">
-        <v>0.03270934581308375</v>
+        <v>0.03270934581308374</v>
       </c>
       <c r="R7">
-        <v>0.0130997380052399</v>
+        <v>0.01309973800523989</v>
       </c>
     </row>
     <row r="8">
@@ -32823,19 +32832,19 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>0.6533034669653304</v>
+        <v>0.6533034669653303</v>
       </c>
       <c r="L10">
         <v>0.1133388666113339</v>
       </c>
       <c r="M10">
-        <v>0.07717922820771793</v>
+        <v>0.07717922820771791</v>
       </c>
       <c r="N10">
-        <v>0.04270957290427096</v>
+        <v>0.04270957290427095</v>
       </c>
       <c r="O10">
-        <v>0.06430935690643096</v>
+        <v>0.06430935690643094</v>
       </c>
       <c r="P10">
         <v>0.02426975730242698</v>
@@ -33116,16 +33125,16 @@
         <v>0.16843</v>
       </c>
       <c r="L15">
-        <v>0.0477</v>
+        <v>0.04770000000000001</v>
       </c>
       <c r="M15">
-        <v>0.07202</v>
+        <v>0.07202000000000001</v>
       </c>
       <c r="N15">
         <v>0.23139</v>
       </c>
       <c r="O15">
-        <v>0.3099</v>
+        <v>0.3099000000000001</v>
       </c>
       <c r="P15">
         <v>0.1333</v>
@@ -33134,7 +33143,7 @@
         <v>0.02852</v>
       </c>
       <c r="R15">
-        <v>0.00874</v>
+        <v>0.008740000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -33229,28 +33238,28 @@
         <v>0</v>
       </c>
       <c r="K17">
-        <v>0.7321126788732112</v>
+        <v>0.7321126788732114</v>
       </c>
       <c r="L17">
-        <v>0.1560084399156008</v>
+        <v>0.1560084399156009</v>
       </c>
       <c r="M17">
         <v>0.03523964760352397</v>
       </c>
       <c r="N17">
-        <v>0.006349936500634993</v>
+        <v>0.006349936500634994</v>
       </c>
       <c r="O17">
         <v>0.01193988060119399</v>
       </c>
       <c r="P17">
-        <v>0.03125968740312597</v>
+        <v>0.03125968740312598</v>
       </c>
       <c r="Q17">
         <v>0.01960980390196098</v>
       </c>
       <c r="R17">
-        <v>0.007479925200747992</v>
+        <v>0.007479925200747993</v>
       </c>
     </row>
     <row r="18">
@@ -33299,10 +33308,10 @@
         <v>0.03353</v>
       </c>
       <c r="O18">
-        <v>0.0098</v>
+        <v>0.009800000000000001</v>
       </c>
       <c r="P18">
-        <v>0.00289</v>
+        <v>0.002890000000000001</v>
       </c>
       <c r="Q18">
         <v>0.01717</v>
@@ -33345,7 +33354,7 @@
         <v>0</v>
       </c>
       <c r="K19">
-        <v>0.69074</v>
+        <v>0.6907399999999999</v>
       </c>
       <c r="L19">
         <v>0.10974</v>
@@ -33354,19 +33363,19 @@
         <v>0.10255</v>
       </c>
       <c r="N19">
-        <v>0.03705</v>
+        <v>0.03704999999999999</v>
       </c>
       <c r="O19">
         <v>0.0153</v>
       </c>
       <c r="P19">
-        <v>0.00709</v>
+        <v>0.007089999999999998</v>
       </c>
       <c r="Q19">
-        <v>0.00682</v>
+        <v>0.006819999999999998</v>
       </c>
       <c r="R19">
-        <v>0.03071</v>
+        <v>0.03070999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -33577,25 +33586,25 @@
         <v>0</v>
       </c>
       <c r="K23">
-        <v>0.7786222137778622</v>
+        <v>0.778622213777862</v>
       </c>
       <c r="L23">
-        <v>0.03435965640343597</v>
+        <v>0.03435965640343596</v>
       </c>
       <c r="M23">
-        <v>0.07256927430725692</v>
+        <v>0.0725692743072569</v>
       </c>
       <c r="N23">
-        <v>0.02962970370296297</v>
+        <v>0.02962970370296296</v>
       </c>
       <c r="O23">
         <v>0.02689973100268997</v>
       </c>
       <c r="P23">
-        <v>0.03224967750322497</v>
+        <v>0.03224967750322496</v>
       </c>
       <c r="Q23">
-        <v>0.01420985790142099</v>
+        <v>0.01420985790142098</v>
       </c>
       <c r="R23">
         <v>0.01145988540114599</v>
@@ -33635,10 +33644,10 @@
         <v>0</v>
       </c>
       <c r="K24">
-        <v>0.04736</v>
+        <v>0.04736000000000001</v>
       </c>
       <c r="L24">
-        <v>0.88844</v>
+        <v>0.8884400000000001</v>
       </c>
       <c r="M24">
         <v>0.02659</v>
@@ -33647,13 +33656,13 @@
         <v>0.02052</v>
       </c>
       <c r="O24">
-        <v>0.009469999999999999</v>
+        <v>0.009470000000000001</v>
       </c>
       <c r="P24">
         <v>0.00217</v>
       </c>
       <c r="Q24">
-        <v>0.00444</v>
+        <v>0.004440000000000001</v>
       </c>
       <c r="R24">
         <v>0.00101</v>
@@ -34206,10 +34215,10 @@
         <v>0.1706017060170602</v>
       </c>
       <c r="K34">
-        <v>0.08509085090850908</v>
+        <v>0.0850908509085091</v>
       </c>
       <c r="L34">
-        <v>0.4347043470434704</v>
+        <v>0.4347043470434705</v>
       </c>
       <c r="M34">
         <v>0.2882128821288213</v>
@@ -34218,7 +34227,7 @@
         <v>0.02004020040200402</v>
       </c>
       <c r="O34">
-        <v>0.001350013500135001</v>
+        <v>0.001350013500135002</v>
       </c>
     </row>
     <row r="35">
@@ -34261,7 +34270,7 @@
         <v>0.24059</v>
       </c>
       <c r="M35">
-        <v>0.60005</v>
+        <v>0.6000500000000001</v>
       </c>
       <c r="N35">
         <v>0.02974</v>
@@ -34399,7 +34408,7 @@
         <v>0</v>
       </c>
       <c r="J38">
-        <v>0.1290912909129091</v>
+        <v>0.1290912909129092</v>
       </c>
       <c r="K38">
         <v>0.7318673186731868</v>
@@ -34414,7 +34423,7 @@
         <v>0.01133011330113301</v>
       </c>
       <c r="O38">
-        <v>0.003300033000330003</v>
+        <v>0.003300033000330004</v>
       </c>
     </row>
     <row r="39">
@@ -34987,10 +34996,10 @@
         <v>0</v>
       </c>
       <c r="J50">
-        <v>0.90094</v>
+        <v>0.9009400000000001</v>
       </c>
       <c r="K50">
-        <v>0.06372999999999999</v>
+        <v>0.06373000000000001</v>
       </c>
       <c r="L50">
         <v>0.01379</v>
@@ -34999,10 +35008,10 @@
         <v>0.0112</v>
       </c>
       <c r="N50">
-        <v>0.00588</v>
+        <v>0.005880000000000001</v>
       </c>
       <c r="O50">
-        <v>0.00446</v>
+        <v>0.004460000000000001</v>
       </c>
     </row>
     <row r="51">
@@ -35036,10 +35045,10 @@
         <v>0</v>
       </c>
       <c r="J51">
-        <v>0.56292</v>
+        <v>0.5629200000000001</v>
       </c>
       <c r="K51">
-        <v>0.38993</v>
+        <v>0.3899300000000001</v>
       </c>
       <c r="L51">
         <v>0.02004</v>
@@ -35048,7 +35057,7 @@
         <v>0.01366</v>
       </c>
       <c r="N51">
-        <v>0.009889999999999999</v>
+        <v>0.009890000000000001</v>
       </c>
       <c r="O51">
         <v>0.00356</v>
@@ -35140,7 +35149,7 @@
         <v>0.2220722207222072</v>
       </c>
       <c r="L53">
-        <v>0.4390743907439074</v>
+        <v>0.4390743907439075</v>
       </c>
       <c r="M53">
         <v>0.2031120311203112</v>
@@ -35281,22 +35290,22 @@
         <v>0</v>
       </c>
       <c r="J56">
-        <v>0.4655</v>
+        <v>0.4654999999999999</v>
       </c>
       <c r="K56">
         <v>0.30824</v>
       </c>
       <c r="L56">
-        <v>0.05659</v>
+        <v>0.05658999999999999</v>
       </c>
       <c r="M56">
-        <v>0.05012</v>
+        <v>0.05011999999999998</v>
       </c>
       <c r="N56">
-        <v>0.07242999999999999</v>
+        <v>0.07242999999999998</v>
       </c>
       <c r="O56">
-        <v>0.04712</v>
+        <v>0.04711999999999999</v>
       </c>
     </row>
     <row r="57">
@@ -35669,7 +35678,7 @@
         <v>0.16689</v>
       </c>
       <c r="J63">
-        <v>0.0251</v>
+        <v>0.02509999999999999</v>
       </c>
       <c r="K63">
         <v>0.18361</v>
@@ -35681,19 +35690,19 @@
         <v>0.13686</v>
       </c>
       <c r="N63">
-        <v>0.08262</v>
+        <v>0.08261999999999999</v>
       </c>
       <c r="O63">
-        <v>0.06088</v>
+        <v>0.06087999999999998</v>
       </c>
       <c r="P63">
-        <v>0.04245</v>
+        <v>0.04244999999999999</v>
       </c>
       <c r="Q63">
-        <v>0.0239</v>
+        <v>0.02389999999999999</v>
       </c>
       <c r="R63">
-        <v>0.02474</v>
+        <v>0.02473999999999999</v>
       </c>
     </row>
     <row r="64">
@@ -35724,16 +35733,16 @@
         <v>54</v>
       </c>
       <c r="I64">
-        <v>0.4194883897677954</v>
+        <v>0.4194883897677953</v>
       </c>
       <c r="J64">
-        <v>0.05925118502370047</v>
+        <v>0.05925118502370046</v>
       </c>
       <c r="K64">
         <v>0.05377107542150843</v>
       </c>
       <c r="L64">
-        <v>0.04102082041640833</v>
+        <v>0.04102082041640832</v>
       </c>
       <c r="M64">
         <v>0.1379527590551811</v>
@@ -35745,13 +35754,13 @@
         <v>0.07389147782955659</v>
       </c>
       <c r="P64">
-        <v>0.03151063021260426</v>
+        <v>0.03151063021260425</v>
       </c>
       <c r="Q64">
         <v>0.01596031920638413</v>
       </c>
       <c r="R64">
-        <v>0.02561051221024421</v>
+        <v>0.0256105122102442</v>
       </c>
     </row>
     <row r="65">
@@ -36072,31 +36081,31 @@
         <v>15</v>
       </c>
       <c r="I70">
-        <v>0.31412</v>
+        <v>0.3141200000000001</v>
       </c>
       <c r="J70">
-        <v>0.00826</v>
+        <v>0.008260000000000002</v>
       </c>
       <c r="K70">
         <v>0.01135</v>
       </c>
       <c r="L70">
-        <v>0.04983</v>
+        <v>0.04983000000000001</v>
       </c>
       <c r="M70">
-        <v>0.52384</v>
+        <v>0.5238400000000001</v>
       </c>
       <c r="N70">
-        <v>0.05053</v>
+        <v>0.05053000000000001</v>
       </c>
       <c r="O70">
         <v>0.03116</v>
       </c>
       <c r="P70">
-        <v>0.008189999999999999</v>
+        <v>0.008190000000000001</v>
       </c>
       <c r="Q70">
-        <v>0.00076</v>
+        <v>0.0007600000000000002</v>
       </c>
       <c r="R70">
         <v>0.00196</v>
@@ -36130,19 +36139,19 @@
         <v>28</v>
       </c>
       <c r="I71">
-        <v>0.2799344013119738</v>
+        <v>0.2799344013119737</v>
       </c>
       <c r="J71">
         <v>0.1622067558648827</v>
       </c>
       <c r="K71">
-        <v>0.05189896202075959</v>
+        <v>0.05189896202075958</v>
       </c>
       <c r="L71">
         <v>0.02363952720945581</v>
       </c>
       <c r="M71">
-        <v>0.01921961560768785</v>
+        <v>0.01921961560768784</v>
       </c>
       <c r="N71">
         <v>0.06021879562408752</v>
@@ -36151,13 +36160,13 @@
         <v>0.3551528969420611</v>
       </c>
       <c r="P71">
-        <v>0.04129917401651968</v>
+        <v>0.04129917401651967</v>
       </c>
       <c r="Q71">
-        <v>0.005709885802283955</v>
+        <v>0.005709885802283953</v>
       </c>
       <c r="R71">
-        <v>0.0007199856002879944</v>
+        <v>0.0007199856002879941</v>
       </c>
     </row>
     <row r="72">
@@ -36249,31 +36258,31 @@
         <v>0.19229</v>
       </c>
       <c r="J73">
-        <v>0.04776</v>
+        <v>0.04776000000000001</v>
       </c>
       <c r="K73">
-        <v>0.30284</v>
+        <v>0.3028400000000001</v>
       </c>
       <c r="L73">
-        <v>0.09919</v>
+        <v>0.09919000000000003</v>
       </c>
       <c r="M73">
-        <v>0.20773</v>
+        <v>0.2077300000000001</v>
       </c>
       <c r="N73">
-        <v>0.09465999999999999</v>
+        <v>0.09466000000000002</v>
       </c>
       <c r="O73">
         <v>0.02021</v>
       </c>
       <c r="P73">
-        <v>0.00817</v>
+        <v>0.008170000000000002</v>
       </c>
       <c r="Q73">
-        <v>0.00633</v>
+        <v>0.006330000000000001</v>
       </c>
       <c r="R73">
-        <v>0.02082</v>
+        <v>0.02082000000000001</v>
       </c>
     </row>
     <row r="74">
@@ -36457,13 +36466,13 @@
         <v>0.3498932006501068</v>
       </c>
       <c r="K77">
-        <v>0.177801958822198</v>
+        <v>0.1778019588221981</v>
       </c>
       <c r="L77">
-        <v>0.06111800893888199</v>
+        <v>0.061118008938882</v>
       </c>
       <c r="M77">
-        <v>0.06520186693479813</v>
+        <v>0.06520186693479814</v>
       </c>
       <c r="N77">
         <v>0.130713966869286</v>
@@ -36552,7 +36561,7 @@
         <v>0</v>
       </c>
       <c r="J79">
-        <v>0.1367648658632351</v>
+        <v>0.1367648658632352</v>
       </c>
       <c r="K79">
         <v>0.1548867828451132</v>
@@ -36561,13 +36570,13 @@
         <v>0.1106557948893442</v>
       </c>
       <c r="M79">
-        <v>0.1677143348322856</v>
+        <v>0.1677143348322857</v>
       </c>
       <c r="N79">
-        <v>0.179696950820303</v>
+        <v>0.1796969508203031</v>
       </c>
       <c r="O79">
-        <v>0.2502812707497187</v>
+        <v>0.2502812707497188</v>
       </c>
     </row>
     <row r="80">
@@ -36696,13 +36705,13 @@
         <v>0</v>
       </c>
       <c r="I82">
-        <v>0.2917886525200027</v>
+        <v>0.2917886525200026</v>
       </c>
       <c r="J82">
-        <v>0.004804855811175865</v>
+        <v>0.004804855811175864</v>
       </c>
       <c r="K82">
-        <v>0.06607635485939325</v>
+        <v>0.06607635485939324</v>
       </c>
       <c r="L82">
         <v>0.4168600099404741</v>
@@ -36711,7 +36720,7 @@
         <v>0.1792314713090655</v>
       </c>
       <c r="N82">
-        <v>0.03020479551425432</v>
+        <v>0.03020479551425431</v>
       </c>
       <c r="O82">
         <v>0.01103386004563431</v>
@@ -36953,19 +36962,19 @@
         <v>0</v>
       </c>
       <c r="J87">
-        <v>0.04473987231240441</v>
+        <v>0.04473987231240443</v>
       </c>
       <c r="K87">
-        <v>0.02039994177856616</v>
+        <v>0.02039994177856617</v>
       </c>
       <c r="L87">
-        <v>0.03759989268990626</v>
+        <v>0.03759989268990627</v>
       </c>
       <c r="M87">
-        <v>0.1032797052397212</v>
+        <v>0.1032797052397213</v>
       </c>
       <c r="N87">
-        <v>0.3393190315834838</v>
+        <v>0.3393190315834839</v>
       </c>
       <c r="O87">
         <v>0.140449599156844</v>
@@ -36974,10 +36983,10 @@
         <v>0.152109565879299</v>
       </c>
       <c r="Q87">
-        <v>0.04825271628674771</v>
+        <v>0.04825271628674772</v>
       </c>
       <c r="R87">
-        <v>0.1138496750730273</v>
+        <v>0.1138496750730274</v>
       </c>
     </row>
     <row r="88">
@@ -37017,13 +37026,13 @@
         <v>0.02791032010346127</v>
       </c>
       <c r="L88">
-        <v>0.08342095675495302</v>
+        <v>0.08342095675495301</v>
       </c>
       <c r="M88">
         <v>0.1167413389064159</v>
       </c>
       <c r="N88">
-        <v>0.08555098118420321</v>
+        <v>0.08555098118420319</v>
       </c>
       <c r="O88">
         <v>0.1021811719158607</v>
@@ -37032,7 +37041,7 @@
         <v>0.2313126529248164</v>
       </c>
       <c r="Q88">
-        <v>0.09436961332509523</v>
+        <v>0.09436961332509522</v>
       </c>
       <c r="R88">
         <v>0.232062661526665</v>
@@ -37075,13 +37084,13 @@
         <v>0.02791032010346127</v>
       </c>
       <c r="L89">
-        <v>0.08342095675495302</v>
+        <v>0.08342095675495301</v>
       </c>
       <c r="M89">
         <v>0.1167413389064159</v>
       </c>
       <c r="N89">
-        <v>0.08555098118420321</v>
+        <v>0.08555098118420319</v>
       </c>
       <c r="O89">
         <v>0.1021811719158607</v>
@@ -37090,7 +37099,7 @@
         <v>0.2313126529248164</v>
       </c>
       <c r="Q89">
-        <v>0.09436961332509523</v>
+        <v>0.09436961332509522</v>
       </c>
       <c r="R89">
         <v>0.232062661526665</v>
@@ -37313,13 +37322,13 @@
         <v>0.09965013193677469</v>
       </c>
       <c r="N93">
-        <v>0.0737600976583693</v>
+        <v>0.07376009765836931</v>
       </c>
       <c r="O93">
-        <v>0.09875013074517311</v>
+        <v>0.09875013074517312</v>
       </c>
       <c r="P93">
-        <v>0.1252301658047395</v>
+        <v>0.1252301658047396</v>
       </c>
       <c r="Q93">
         <v>0.1844589202236104</v>
@@ -37417,7 +37426,7 @@
         <v>0.009290050073369895</v>
       </c>
       <c r="J95">
-        <v>0.07435040074866003</v>
+        <v>0.07435040074866002</v>
       </c>
       <c r="K95">
         <v>0.1840109918192459</v>
@@ -37426,7 +37435,7 @@
         <v>0.1933110419465161</v>
       </c>
       <c r="M95">
-        <v>0.1487008014973201</v>
+        <v>0.14870080149732</v>
       </c>
       <c r="N95">
         <v>0.117100631172402</v>
@@ -37435,13 +37444,13 @@
         <v>0.1059505710735781</v>
       </c>
       <c r="P95">
-        <v>0.07063038069775196</v>
+        <v>0.07063038069775195</v>
       </c>
       <c r="Q95">
         <v>0.04461024044919602</v>
       </c>
       <c r="R95">
-        <v>0.05204489052195991</v>
+        <v>0.0520448905219599</v>
       </c>
     </row>
     <row r="96">
@@ -37786,10 +37795,10 @@
         <v>0.1942609975302223</v>
       </c>
       <c r="Q101">
-        <v>0.08277042502613251</v>
+        <v>0.08277042502613249</v>
       </c>
       <c r="R101">
-        <v>0.05236513389496255</v>
+        <v>0.05236513389496254</v>
       </c>
     </row>
     <row r="102">
@@ -37881,31 +37890,31 @@
         <v>0</v>
       </c>
       <c r="J103">
-        <v>0.06532965969780263</v>
+        <v>0.06532965969780262</v>
       </c>
       <c r="K103">
-        <v>0.02344987784958628</v>
+        <v>0.02344987784958627</v>
       </c>
       <c r="L103">
-        <v>0.02177988654857097</v>
+        <v>0.02177988654857096</v>
       </c>
       <c r="M103">
         <v>0.1004994764982269</v>
       </c>
       <c r="N103">
-        <v>0.5929569112874491</v>
+        <v>0.592956911287449</v>
       </c>
       <c r="O103">
-        <v>0.1356792932465615</v>
+        <v>0.1356792932465614</v>
       </c>
       <c r="P103">
-        <v>0.04689975569917256</v>
+        <v>0.04689975569917255</v>
       </c>
       <c r="Q103">
-        <v>0.005029973798866482</v>
+        <v>0.00502997379886648</v>
       </c>
       <c r="R103">
-        <v>0.008375165373763567</v>
+        <v>0.008375165373763566</v>
       </c>
     </row>
     <row r="104">
@@ -38052,7 +38061,7 @@
         <v>0</v>
       </c>
       <c r="I106">
-        <v>0.03672036720367203</v>
+        <v>0.03672036720367204</v>
       </c>
       <c r="J106">
         <v>0.03011030110301103</v>
@@ -38591,7 +38600,7 @@
         <v>0</v>
       </c>
       <c r="I117">
-        <v>0.002930029300293003</v>
+        <v>0.002930029300293002</v>
       </c>
       <c r="J117">
         <v>0.1123311233112331</v>
@@ -38609,7 +38618,7 @@
         <v>0.2108121081210812</v>
       </c>
       <c r="O117">
-        <v>0.2363223632236323</v>
+        <v>0.2363223632236322</v>
       </c>
     </row>
     <row r="118">
@@ -38842,7 +38851,7 @@
         <v>0.06145061450614506</v>
       </c>
       <c r="K122">
-        <v>0.04571045710457104</v>
+        <v>0.04571045710457105</v>
       </c>
       <c r="L122">
         <v>0.05234052340523405</v>
@@ -38851,7 +38860,7 @@
         <v>0.1310013100131001</v>
       </c>
       <c r="N122">
-        <v>0.2242322423224232</v>
+        <v>0.2242322423224233</v>
       </c>
       <c r="O122">
         <v>0.4748147481474815</v>
@@ -38940,7 +38949,7 @@
         <v>0.04103</v>
       </c>
       <c r="K124">
-        <v>0.08898</v>
+        <v>0.08898000000000002</v>
       </c>
       <c r="L124">
         <v>0.15433</v>
@@ -39179,7 +39188,7 @@
         <v>210</v>
       </c>
       <c r="I129">
-        <v>0.9031090310903108</v>
+        <v>0.9031090310903109</v>
       </c>
       <c r="J129">
         <v>0.01050010500105001</v>
@@ -39188,7 +39197,7 @@
         <v>0.04249042490424904</v>
       </c>
       <c r="L129">
-        <v>0.006610066100661007</v>
+        <v>0.006610066100661008</v>
       </c>
       <c r="M129">
         <v>0.008340083400834008</v>
@@ -39197,7 +39206,7 @@
         <v>0.01234012340123401</v>
       </c>
       <c r="O129">
-        <v>0.009720097200972009</v>
+        <v>0.00972009720097201</v>
       </c>
       <c r="P129">
         <v>0.004420044200442005</v>
@@ -39237,7 +39246,7 @@
         <v>222</v>
       </c>
       <c r="I130">
-        <v>0.001820018200182002</v>
+        <v>0.001820018200182001</v>
       </c>
       <c r="J130">
         <v>0.06383063830638305</v>
@@ -39255,10 +39264,10 @@
         <v>0.01115011150111501</v>
       </c>
       <c r="O130">
-        <v>0.005090050900509005</v>
+        <v>0.005090050900509004</v>
       </c>
       <c r="P130">
-        <v>0.005160051600516005</v>
+        <v>0.005160051600516004</v>
       </c>
       <c r="Q130">
         <v>0.003680036800368003</v>
@@ -39411,31 +39420,31 @@
         <v>122</v>
       </c>
       <c r="I133">
-        <v>0.8408100000000001</v>
+        <v>0.8408100000000003</v>
       </c>
       <c r="J133">
         <v>0.03148000000000001</v>
       </c>
       <c r="K133">
-        <v>0.05280000000000001</v>
+        <v>0.05280000000000002</v>
       </c>
       <c r="L133">
-        <v>0.05046</v>
+        <v>0.05046000000000001</v>
       </c>
       <c r="M133">
-        <v>0.007180000000000001</v>
+        <v>0.007180000000000002</v>
       </c>
       <c r="N133">
-        <v>0.0008900000000000001</v>
+        <v>0.0008900000000000003</v>
       </c>
       <c r="O133">
-        <v>0.0007900000000000001</v>
+        <v>0.0007900000000000002</v>
       </c>
       <c r="P133">
         <v>0.002560000000000001</v>
       </c>
       <c r="Q133">
-        <v>0.008530000000000001</v>
+        <v>0.008530000000000003</v>
       </c>
       <c r="R133">
         <v>0.004500000000000001</v>
@@ -39674,13 +39683,13 @@
         <v>0</v>
       </c>
       <c r="I138">
-        <v>0.8408668408668409</v>
+        <v>0.8408668408668408</v>
       </c>
       <c r="J138">
         <v>0.03881303881303881</v>
       </c>
       <c r="K138">
-        <v>0.06928406928406929</v>
+        <v>0.06928406928406927</v>
       </c>
       <c r="L138">
         <v>0.02576702576702577</v>
@@ -39689,7 +39698,7 @@
         <v>0.01528301528301528</v>
       </c>
       <c r="N138">
-        <v>0.008631008631008632</v>
+        <v>0.00863100863100863</v>
       </c>
       <c r="O138">
         <v>0.001355001355001355</v>
@@ -39891,22 +39900,22 @@
         <v>0.00023</v>
       </c>
       <c r="J142">
-        <v>0.0357</v>
+        <v>0.03570000000000001</v>
       </c>
       <c r="K142">
-        <v>0.06007</v>
+        <v>0.06007000000000001</v>
       </c>
       <c r="L142">
         <v>0.13767</v>
       </c>
       <c r="M142">
-        <v>0.52208</v>
+        <v>0.5220800000000001</v>
       </c>
       <c r="N142">
         <v>0.15082</v>
       </c>
       <c r="O142">
-        <v>0.05655</v>
+        <v>0.05655000000000001</v>
       </c>
       <c r="P142">
         <v>0.01469</v>
@@ -39915,7 +39924,7 @@
         <v>0.01298</v>
       </c>
       <c r="R142">
-        <v>0.009209999999999999</v>
+        <v>0.009210000000000001</v>
       </c>
     </row>
     <row r="143">
@@ -39949,7 +39958,7 @@
         <v>0.00186</v>
       </c>
       <c r="J143">
-        <v>0.06586</v>
+        <v>0.06586000000000002</v>
       </c>
       <c r="K143">
         <v>0.20998</v>
@@ -39961,13 +39970,13 @@
         <v>0.14708</v>
       </c>
       <c r="N143">
-        <v>0.28513</v>
+        <v>0.2851300000000001</v>
       </c>
       <c r="O143">
-        <v>0.08232</v>
+        <v>0.08232000000000002</v>
       </c>
       <c r="P143">
-        <v>0.03497</v>
+        <v>0.03497000000000001</v>
       </c>
       <c r="Q143">
         <v>0.01302</v>
@@ -40004,7 +40013,7 @@
         <v>200</v>
       </c>
       <c r="I144">
-        <v>0.0004900049000490004</v>
+        <v>0.0004900049000490005</v>
       </c>
       <c r="J144">
         <v>0.01794017940179402</v>
@@ -40013,10 +40022,10 @@
         <v>0.2824928249282493</v>
       </c>
       <c r="L144">
-        <v>0.4622146221462214</v>
+        <v>0.4622146221462215</v>
       </c>
       <c r="M144">
-        <v>0.07363073630736307</v>
+        <v>0.07363073630736308</v>
       </c>
       <c r="N144">
         <v>0.04897048970489705</v>
@@ -40031,7 +40040,7 @@
         <v>0.01201012010120101</v>
       </c>
       <c r="R144">
-        <v>0.004450044500445004</v>
+        <v>0.004450044500445005</v>
       </c>
     </row>
     <row r="145">
@@ -40062,28 +40071,28 @@
         <v>200</v>
       </c>
       <c r="I145">
-        <v>0.00271</v>
+        <v>0.002710000000000001</v>
       </c>
       <c r="J145">
-        <v>0.05448</v>
+        <v>0.05448000000000001</v>
       </c>
       <c r="K145">
         <v>0.15424</v>
       </c>
       <c r="L145">
-        <v>0.32356</v>
+        <v>0.3235600000000001</v>
       </c>
       <c r="M145">
         <v>0.23351</v>
       </c>
       <c r="N145">
-        <v>0.07711</v>
+        <v>0.07711000000000001</v>
       </c>
       <c r="O145">
-        <v>0.0596</v>
+        <v>0.05960000000000001</v>
       </c>
       <c r="P145">
-        <v>0.05423</v>
+        <v>0.05423000000000001</v>
       </c>
       <c r="Q145">
         <v>0.02743</v>
@@ -40126,13 +40135,13 @@
         <v>0.02256977430225698</v>
       </c>
       <c r="K146">
-        <v>0.1657683423165768</v>
+        <v>0.1657683423165769</v>
       </c>
       <c r="L146">
-        <v>0.3434665653343466</v>
+        <v>0.3434665653343467</v>
       </c>
       <c r="M146">
-        <v>0.2758472415275847</v>
+        <v>0.2758472415275848</v>
       </c>
       <c r="N146">
         <v>0.1096489035109649</v>
@@ -40147,7 +40156,7 @@
         <v>0.01949980500194998</v>
       </c>
       <c r="R146">
-        <v>0.003189968100318997</v>
+        <v>0.003189968100318998</v>
       </c>
     </row>
     <row r="147">
@@ -40413,7 +40422,7 @@
         <v>0.01198</v>
       </c>
       <c r="J151">
-        <v>0.07269</v>
+        <v>0.07269000000000002</v>
       </c>
       <c r="K151">
         <v>0.17624</v>
@@ -40425,7 +40434,7 @@
         <v>0.23362</v>
       </c>
       <c r="N151">
-        <v>0.09937</v>
+        <v>0.09937000000000001</v>
       </c>
       <c r="O151">
         <v>0.10827</v>
@@ -40434,10 +40443,10 @@
         <v>0.13094</v>
       </c>
       <c r="Q151">
-        <v>0.0523</v>
+        <v>0.05230000000000001</v>
       </c>
       <c r="R151">
-        <v>0.0089</v>
+        <v>0.008900000000000002</v>
       </c>
     </row>
     <row r="152">
@@ -40663,13 +40672,13 @@
         <v>0.16778</v>
       </c>
       <c r="P155">
-        <v>0.09507</v>
+        <v>0.09507000000000002</v>
       </c>
       <c r="Q155">
         <v>0.02296</v>
       </c>
       <c r="R155">
-        <v>0.0385</v>
+        <v>0.03850000000000001</v>
       </c>
     </row>
     <row r="156">
@@ -40706,22 +40715,22 @@
         <v>0.01232987670123299</v>
       </c>
       <c r="K156">
-        <v>0.08782912170878292</v>
+        <v>0.08782912170878293</v>
       </c>
       <c r="L156">
-        <v>0.04704952950470495</v>
+        <v>0.04704952950470496</v>
       </c>
       <c r="M156">
-        <v>0.04147958520414796</v>
+        <v>0.04147958520414797</v>
       </c>
       <c r="N156">
-        <v>0.08002919970800292</v>
+        <v>0.08002919970800294</v>
       </c>
       <c r="O156">
-        <v>0.3678863211367886</v>
+        <v>0.3678863211367887</v>
       </c>
       <c r="P156">
-        <v>0.04061959380406196</v>
+        <v>0.04061959380406197</v>
       </c>
       <c r="Q156">
         <v>0.2072479275207248</v>
@@ -40764,7 +40773,7 @@
         <v>0.01513</v>
       </c>
       <c r="K157">
-        <v>0.03218</v>
+        <v>0.03218000000000001</v>
       </c>
       <c r="L157">
         <v>0.20506</v>
@@ -40776,13 +40785,13 @@
         <v>0.11496</v>
       </c>
       <c r="O157">
-        <v>0.08327</v>
+        <v>0.08327000000000001</v>
       </c>
       <c r="P157">
         <v>0.17259</v>
       </c>
       <c r="Q157">
-        <v>0.05289</v>
+        <v>0.05289000000000001</v>
       </c>
       <c r="R157">
         <v>0.10442</v>
@@ -41106,7 +41115,7 @@
         <v>167</v>
       </c>
       <c r="I163">
-        <v>0.00421</v>
+        <v>0.004209999999999999</v>
       </c>
       <c r="J163">
         <v>0.00146</v>
@@ -41115,19 +41124,19 @@
         <v>0.1467</v>
       </c>
       <c r="L163">
-        <v>0.25061</v>
+        <v>0.2506099999999999</v>
       </c>
       <c r="M163">
         <v>0.11009</v>
       </c>
       <c r="N163">
-        <v>0.06496</v>
+        <v>0.06495999999999999</v>
       </c>
       <c r="O163">
-        <v>0.07381</v>
+        <v>0.07380999999999999</v>
       </c>
       <c r="P163">
-        <v>0.08601</v>
+        <v>0.08600999999999999</v>
       </c>
       <c r="Q163">
         <v>0.12501</v>
@@ -41286,7 +41295,7 @@
         <v>0.1403914039140391</v>
       </c>
       <c r="K166">
-        <v>0.0913109131091311</v>
+        <v>0.09131091310913109</v>
       </c>
       <c r="L166">
         <v>0.1017210172101721</v>
@@ -41295,7 +41304,7 @@
         <v>0.1305213052130521</v>
       </c>
       <c r="N166">
-        <v>0.1744717447174472</v>
+        <v>0.1744717447174471</v>
       </c>
       <c r="O166">
         <v>0.2001120011200112</v>
@@ -41304,7 +41313,7 @@
         <v>0.06552065520655206</v>
       </c>
       <c r="Q166">
-        <v>0.03745037450374504</v>
+        <v>0.03745037450374503</v>
       </c>
       <c r="R166">
         <v>0.04830048300483005</v>
@@ -41399,25 +41408,25 @@
         <v>0.00211</v>
       </c>
       <c r="J168">
-        <v>0.03968</v>
+        <v>0.03968000000000001</v>
       </c>
       <c r="K168">
-        <v>0.31673</v>
+        <v>0.3167300000000001</v>
       </c>
       <c r="L168">
-        <v>0.33854</v>
+        <v>0.3385400000000001</v>
       </c>
       <c r="M168">
-        <v>0.07856</v>
+        <v>0.07856000000000002</v>
       </c>
       <c r="N168">
         <v>0.04801</v>
       </c>
       <c r="O168">
-        <v>0.0687</v>
+        <v>0.06870000000000001</v>
       </c>
       <c r="P168">
-        <v>0.05545</v>
+        <v>0.05545000000000001</v>
       </c>
       <c r="Q168">
         <v>0.03811</v>
@@ -41570,25 +41579,25 @@
         <v>233</v>
       </c>
       <c r="I171">
-        <v>0.03279</v>
+        <v>0.03279000000000001</v>
       </c>
       <c r="J171">
         <v>0.11588</v>
       </c>
       <c r="K171">
-        <v>0.06191</v>
+        <v>0.06191000000000001</v>
       </c>
       <c r="L171">
-        <v>0.04089</v>
+        <v>0.04089000000000001</v>
       </c>
       <c r="M171">
-        <v>0.08878</v>
+        <v>0.08878000000000001</v>
       </c>
       <c r="N171">
-        <v>0.40737</v>
+        <v>0.4073700000000001</v>
       </c>
       <c r="O171">
-        <v>0.19036</v>
+        <v>0.1903600000000001</v>
       </c>
       <c r="P171">
         <v>0.03641</v>
@@ -41637,10 +41646,10 @@
         <v>0.1364127282545651</v>
       </c>
       <c r="L172">
-        <v>0.04594091881837637</v>
+        <v>0.04594091881837638</v>
       </c>
       <c r="M172">
-        <v>0.04231084621692434</v>
+        <v>0.04231084621692435</v>
       </c>
       <c r="N172">
         <v>0.06555131102622053</v>
@@ -41652,7 +41661,7 @@
         <v>0.122482449648993</v>
       </c>
       <c r="Q172">
-        <v>0.02909058181163623</v>
+        <v>0.02909058181163624</v>
       </c>
       <c r="R172">
         <v>0.01122022440448809</v>
@@ -41878,13 +41887,13 @@
         <v>0.16319</v>
       </c>
       <c r="O176">
-        <v>0.03698</v>
+        <v>0.03698000000000001</v>
       </c>
       <c r="P176">
-        <v>0.00759</v>
+        <v>0.007590000000000001</v>
       </c>
       <c r="Q176">
-        <v>0.00478</v>
+        <v>0.004780000000000001</v>
       </c>
       <c r="R176">
         <v>0.01225</v>
@@ -41976,31 +41985,31 @@
         <v>159</v>
       </c>
       <c r="I178">
-        <v>0.008389916100838991</v>
+        <v>0.008389916100838992</v>
       </c>
       <c r="J178">
         <v>0.03896961030389696</v>
       </c>
       <c r="K178">
-        <v>0.1473485265147348</v>
+        <v>0.1473485265147349</v>
       </c>
       <c r="L178">
-        <v>0.07665923340766592</v>
+        <v>0.07665923340766594</v>
       </c>
       <c r="M178">
         <v>0.1877981220187798</v>
       </c>
       <c r="N178">
-        <v>0.2481775182248177</v>
+        <v>0.2481775182248178</v>
       </c>
       <c r="O178">
-        <v>0.1815381846181538</v>
+        <v>0.1815381846181539</v>
       </c>
       <c r="P178">
-        <v>0.07412925870741292</v>
+        <v>0.07412925870741294</v>
       </c>
       <c r="Q178">
-        <v>0.01454985450145498</v>
+        <v>0.01454985450145499</v>
       </c>
       <c r="R178">
         <v>0.02243977560224398</v>
@@ -42034,10 +42043,10 @@
         <v>261</v>
       </c>
       <c r="I179">
-        <v>0.00061</v>
+        <v>0.0006100000000000001</v>
       </c>
       <c r="J179">
-        <v>0.08371000000000001</v>
+        <v>0.08371000000000002</v>
       </c>
       <c r="K179">
         <v>0.05361</v>
@@ -42046,7 +42055,7 @@
         <v>0.25053</v>
       </c>
       <c r="M179">
-        <v>0.0969</v>
+        <v>0.09690000000000001</v>
       </c>
       <c r="N179">
         <v>0.11961</v>
@@ -42058,7 +42067,7 @@
         <v>0.1402</v>
       </c>
       <c r="Q179">
-        <v>0.05521</v>
+        <v>0.05521000000000001</v>
       </c>
       <c r="R179">
         <v>0.02484</v>
@@ -42098,28 +42107,28 @@
         <v>0.04148958510414896</v>
       </c>
       <c r="K180">
-        <v>0.5188548114518854</v>
+        <v>0.5188548114518855</v>
       </c>
       <c r="L180">
-        <v>0.07406925930740692</v>
+        <v>0.07406925930740693</v>
       </c>
       <c r="M180">
-        <v>0.1552184478155218</v>
+        <v>0.1552184478155219</v>
       </c>
       <c r="N180">
         <v>0.04834951650483495</v>
       </c>
       <c r="O180">
-        <v>0.05924940750592493</v>
+        <v>0.05924940750592494</v>
       </c>
       <c r="P180">
-        <v>0.05777942220577793</v>
+        <v>0.05777942220577795</v>
       </c>
       <c r="Q180">
-        <v>0.02798972010279897</v>
+        <v>0.02798972010279898</v>
       </c>
       <c r="R180">
-        <v>0.01699983000169998</v>
+        <v>0.01699983000169999</v>
       </c>
     </row>
     <row r="181">
@@ -42153,28 +42162,28 @@
         <v>0</v>
       </c>
       <c r="J181">
-        <v>0.004219957800421995</v>
+        <v>0.004219957800421996</v>
       </c>
       <c r="K181">
-        <v>0.05050949490505095</v>
+        <v>0.05050949490505096</v>
       </c>
       <c r="L181">
-        <v>0.862241377586224</v>
+        <v>0.8622413775862242</v>
       </c>
       <c r="M181">
-        <v>0.03531964680353196</v>
+        <v>0.03531964680353197</v>
       </c>
       <c r="N181">
         <v>0.03390966090339097</v>
       </c>
       <c r="O181">
-        <v>0.007659923400765992</v>
+        <v>0.007659923400765994</v>
       </c>
       <c r="P181">
-        <v>0.003559964400355996</v>
+        <v>0.003559964400355997</v>
       </c>
       <c r="Q181">
-        <v>0.001499985000149998</v>
+        <v>0.001499985000149999</v>
       </c>
       <c r="R181">
         <v>0.001079989200107999</v>
@@ -42672,7 +42681,7 @@
         <v>0.0106</v>
       </c>
       <c r="K190">
-        <v>0.05913</v>
+        <v>0.05913000000000001</v>
       </c>
       <c r="L190">
         <v>0.41967</v>
@@ -42681,13 +42690,13 @@
         <v>0.41677</v>
       </c>
       <c r="N190">
-        <v>0.08964999999999999</v>
+        <v>0.08965000000000001</v>
       </c>
       <c r="O190">
-        <v>0.00386</v>
+        <v>0.003860000000000001</v>
       </c>
       <c r="P190">
-        <v>0.00032</v>
+        <v>0.0003200000000000001</v>
       </c>
     </row>
     <row r="191">
@@ -42727,10 +42736,10 @@
         <v>0.01728017280172802</v>
       </c>
       <c r="L191">
-        <v>0.1686316863168631</v>
+        <v>0.1686316863168632</v>
       </c>
       <c r="M191">
-        <v>0.4702347023470234</v>
+        <v>0.4702347023470235</v>
       </c>
       <c r="N191">
         <v>0.2593525935259353</v>
@@ -42941,7 +42950,7 @@
         <v>0.4241</v>
       </c>
       <c r="N195">
-        <v>0.08105</v>
+        <v>0.08105000000000001</v>
       </c>
       <c r="O195">
         <v>0.01372</v>
@@ -42981,19 +42990,19 @@
         <v>0</v>
       </c>
       <c r="J196">
-        <v>0.00417</v>
+        <v>0.004170000000000001</v>
       </c>
       <c r="K196">
         <v>0.17917</v>
       </c>
       <c r="L196">
-        <v>0.45833</v>
+        <v>0.4583300000000001</v>
       </c>
       <c r="M196">
-        <v>0.3175</v>
+        <v>0.3175000000000001</v>
       </c>
       <c r="N196">
-        <v>0.03833</v>
+        <v>0.03833000000000001</v>
       </c>
       <c r="O196">
         <v>0.0025</v>

</xml_diff>